<commit_message>
Kanalliste: YouTube-Links in Excel anklickbar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U8rX9WoPvch1isV4z66GEi
</commit_message>
<xml_diff>
--- a/recherche/youtube-kanaele-podcast-gaeste.xlsx
+++ b/recherche/youtube-kanaele-podcast-gaeste.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +31,15 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="4">
@@ -63,10 +72,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,152 +480,146 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>YouTube-Link (anklickbar)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>E-Mail</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Weitere Kontakte</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Themen</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Kategorie</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>20–60k</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Angefragt am</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Notizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Wolf-Dieter Storl</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Dr. Wolf-Dieter Storl</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>287.000</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@wdstorl</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>– (über Website/Verlag prüfen)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>storl.de</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pflanzen, Schamanismus, Germanen, Naturmystik</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Nordisch &amp; Heidentum</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Benjamin Maier</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Schamane Benjamin Maier</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>89.200</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@schamanebenjamin</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>– (über Website prüfen)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>E-Mail</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Weitere Kontakte</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Themen</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Kategorie</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>20–60k</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Angefragt am</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Notizen</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Wolf-Dieter Storl</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Dr. Wolf-Dieter Storl</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>287.000</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@wdstorl</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>– (über Website/Verlag prüfen)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>storl.de</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Pflanzen, Schamanismus, Germanen, Naturmystik</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Schamanismus, Spiritualität</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Nordisch &amp; Heidentum</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Benjamin Maier</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Schamane Benjamin Maier</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>89.200</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@schamanebenjamin</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>– (über Website prüfen)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Schamanismus, Spiritualität</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Nordisch &amp; Heidentum</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Kaptorga - Visual History</t>
         </is>
@@ -627,7 +634,7 @@
           <t>42.400</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@KaptorgaVisualHistory</t>
         </is>
@@ -666,7 +673,7 @@
       <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Heiden TV</t>
         </is>
@@ -681,7 +688,7 @@
           <t>26.500</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@HeidenTV</t>
         </is>
@@ -720,7 +727,7 @@
       <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Richard der weiße Wolf</t>
         </is>
@@ -735,7 +742,7 @@
           <t>11.000</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Richard-der-weiße-wolf</t>
         </is>
@@ -760,17 +767,14 @@
           <t>Nordisch &amp; Heidentum</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Geheimnisakademie - Runen</t>
         </is>
@@ -785,7 +789,7 @@
           <t>8.530</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Geheimnisakademie-Runen</t>
         </is>
@@ -810,17 +814,14 @@
           <t>Nordisch &amp; Heidentum</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Allsherjargode</t>
         </is>
@@ -835,7 +836,7 @@
           <t>5.920</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@allsherjargode</t>
         </is>
@@ -860,17 +861,14 @@
           <t>Nordisch &amp; Heidentum</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>MYSTICA Magazin</t>
         </is>
@@ -885,7 +883,7 @@
           <t>151.000</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@mysticatv</t>
         </is>
@@ -910,17 +908,14 @@
           <t>Mystik &amp; Grenzwissen</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>ExoMagazinTV</t>
         </is>
@@ -935,7 +930,7 @@
           <t>149.000</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@ExoMagazinTV</t>
         </is>
@@ -960,17 +955,14 @@
           <t>Mystik &amp; Grenzwissen</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Chnopfloch</t>
         </is>
@@ -985,7 +977,7 @@
           <t>97.000</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Chnopfloch</t>
         </is>
@@ -1010,17 +1002,14 @@
           <t>Mystik &amp; Grenzwissen</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Hangar18b</t>
         </is>
@@ -1035,7 +1024,7 @@
           <t>46.400</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Hangar18b</t>
         </is>
@@ -1074,7 +1063,7 @@
       <c r="L12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Thomas Ritter</t>
         </is>
@@ -1089,7 +1078,7 @@
           <t>41.900</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@thomasritter1811</t>
         </is>
@@ -1128,7 +1117,7 @@
       <c r="L13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Tarastro</t>
         </is>
@@ -1143,7 +1132,7 @@
           <t>37.300</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@tarastro3500</t>
         </is>
@@ -1182,7 +1171,7 @@
       <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>XXMIGOO</t>
         </is>
@@ -1197,7 +1186,7 @@
           <t>31.500</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@XXMIGOO</t>
         </is>
@@ -1236,7 +1225,7 @@
       <c r="L15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Phioo wills wissen</t>
         </is>
@@ -1251,7 +1240,7 @@
           <t>22.100</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Phioowillswissen</t>
         </is>
@@ -1290,7 +1279,7 @@
       <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Sagenhaft und Sonderbar (Podcast)</t>
         </is>
@@ -1305,7 +1294,7 @@
           <t>14.300</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@sagenhaftundsonderbar</t>
         </is>
@@ -1330,17 +1319,14 @@
           <t>Mystik &amp; Grenzwissen</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Salvatore Princi</t>
         </is>
@@ -1355,7 +1341,7 @@
           <t>57.400</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@salvatoreprinci</t>
         </is>
@@ -1394,7 +1380,7 @@
       <c r="L18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>REAL. by Jens Lehrich</t>
         </is>
@@ -1409,7 +1395,7 @@
           <t>42.200</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@jens-lehrich</t>
         </is>
@@ -1448,7 +1434,7 @@
       <c r="L19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Human Elevation Podcast</t>
         </is>
@@ -1463,7 +1449,7 @@
           <t>37.100</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Human_Elevation_Podcast</t>
         </is>
@@ -1502,7 +1488,7 @@
       <c r="L20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Burchardt &amp; Böttcher</t>
         </is>
@@ -1517,7 +1503,7 @@
           <t>37.100</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@burchardtundboettcher</t>
         </is>
@@ -1556,7 +1542,7 @@
       <c r="L21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Andreas Goldemann</t>
         </is>
@@ -1571,7 +1557,7 @@
           <t>26.900</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@AndreasGoldemann</t>
         </is>
@@ -1610,7 +1596,7 @@
       <c r="L22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Deine Seelenreise</t>
         </is>
@@ -1625,7 +1611,7 @@
           <t>26.900</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Deineseelenreise8</t>
         </is>
@@ -1664,7 +1650,7 @@
       <c r="L23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Dodefi</t>
         </is>
@@ -1679,7 +1665,7 @@
           <t>23.000</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Dodefi-Podcast</t>
         </is>
@@ -1718,7 +1704,7 @@
       <c r="L24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Matrixwissen</t>
         </is>
@@ -1733,7 +1719,7 @@
           <t>22.700</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Matrixwissen</t>
         </is>
@@ -1772,7 +1758,7 @@
       <c r="L25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>aufge-wacht by Liv Wach</t>
         </is>
@@ -1787,7 +1773,7 @@
           <t>22.100</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@aufge-wachtbylivwach</t>
         </is>
@@ -1826,7 +1812,7 @@
       <c r="L26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Armin Risi</t>
         </is>
@@ -1841,7 +1827,7 @@
           <t>18.600</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@RisiArmin</t>
         </is>
@@ -1866,17 +1852,14 @@
           <t>Bewusstsein &amp; Matrix</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Matrixxer</t>
         </is>
@@ -1891,7 +1874,7 @@
           <t>12.400</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Matrixxer</t>
         </is>
@@ -1916,17 +1899,14 @@
           <t>Bewusstsein &amp; Matrix</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>My Big TOE auf Deutsch</t>
         </is>
@@ -1941,7 +1921,7 @@
           <t>12.000</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@MyBigTOEaufDeutsch</t>
         </is>
@@ -1966,17 +1946,14 @@
           <t>Bewusstsein &amp; Matrix</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>BETZ BEWEGT</t>
         </is>
@@ -1991,7 +1968,7 @@
           <t>272.000</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@RobertBetzTV</t>
         </is>
@@ -2016,17 +1993,14 @@
           <t>Bewusstsein &amp; Spiritualität</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Christina von Dreien</t>
         </is>
@@ -2041,7 +2015,7 @@
           <t>165.000</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Christina-Von-Dreien</t>
         </is>
@@ -2066,17 +2040,14 @@
           <t>Bewusstsein &amp; Spiritualität</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Pierre Franckh</t>
         </is>
@@ -2091,7 +2062,7 @@
           <t>140.000</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@PierreFranckh</t>
         </is>
@@ -2116,17 +2087,14 @@
           <t>Bewusstsein &amp; Spiritualität</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Dieter Broers</t>
         </is>
@@ -2141,7 +2109,7 @@
           <t>139.000</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@dieterbroersnow</t>
         </is>
@@ -2166,17 +2134,14 @@
           <t>Bewusstsein &amp; Spiritualität</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>dieZuversicht</t>
         </is>
@@ -2191,7 +2156,7 @@
           <t>98.700</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@dieZuversicht</t>
         </is>
@@ -2216,17 +2181,14 @@
           <t>Bewusstsein &amp; Spiritualität</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Gerald Hüther</t>
         </is>
@@ -2241,7 +2203,7 @@
           <t>78.000</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@GeraldHuether-original</t>
         </is>
@@ -2266,17 +2228,14 @@
           <t>Bewusstsein &amp; Spiritualität</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>Ruediger Dahlke</t>
         </is>
@@ -2291,7 +2250,7 @@
           <t>44.400</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@RuedigerDahlke</t>
         </is>
@@ -2330,7 +2289,7 @@
       <c r="L36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Frank Köstler</t>
         </is>
@@ -2345,7 +2304,7 @@
           <t>28.100</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@frankkoestler1510</t>
         </is>
@@ -2384,7 +2343,7 @@
       <c r="L37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>Jo Conrad / Bewusst.TV</t>
         </is>
@@ -2399,7 +2358,7 @@
           <t>10.100</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@joconrad3789</t>
         </is>
@@ -2424,17 +2383,14 @@
           <t>Bewusstsein &amp; Spiritualität</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Daniele Ganser</t>
         </is>
@@ -2449,7 +2405,7 @@
           <t>506.000</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@DanieleGanserOffiziell</t>
         </is>
@@ -2474,17 +2430,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>Hoss &amp; Hopf</t>
         </is>
@@ -2499,7 +2452,7 @@
           <t>418.000</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@hoss_und_hopf</t>
         </is>
@@ -2524,17 +2477,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>QS24</t>
         </is>
@@ -2549,7 +2499,7 @@
           <t>392.000</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@QS24</t>
         </is>
@@ -2574,17 +2524,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>Jasmin Kosubek</t>
         </is>
@@ -2599,7 +2546,7 @@
           <t>352.000</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@JasminKosubekOriginal</t>
         </is>
@@ -2624,17 +2571,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>NuoViso</t>
         </is>
@@ -2649,7 +2593,7 @@
           <t>275.000</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@NuoVisoTv</t>
         </is>
@@ -2674,17 +2618,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>Fair Talk</t>
         </is>
@@ -2699,7 +2640,7 @@
           <t>250.000</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@FAIRTALKTV</t>
         </is>
@@ -2724,17 +2665,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>LION Media</t>
         </is>
@@ -2749,7 +2687,7 @@
           <t>211.000</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@LIONMediaNews</t>
         </is>
@@ -2774,17 +2712,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>Wissensmanufaktur</t>
         </is>
@@ -2799,7 +2734,7 @@
           <t>207.000</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@wissensmanufaktur</t>
         </is>
@@ -2824,17 +2759,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>NachDenkSeiten</t>
         </is>
@@ -2849,7 +2781,7 @@
           <t>191.000</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@nachdenkseiten745</t>
         </is>
@@ -2874,17 +2806,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>Hallo Meinung</t>
         </is>
@@ -2899,7 +2828,7 @@
           <t>176.000</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@HalloMeinung</t>
         </is>
@@ -2924,17 +2853,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>SchrangTV</t>
         </is>
@@ -2949,7 +2875,7 @@
           <t>172.000</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@SchrangTV</t>
         </is>
@@ -2974,17 +2900,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>eingeSCHENKt.tv</t>
         </is>
@@ -2999,7 +2922,7 @@
           <t>170.000</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@eingeSCHENKTtv</t>
         </is>
@@ -3024,17 +2947,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>NuoFlix</t>
         </is>
@@ -3049,7 +2969,7 @@
           <t>158.000</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@nuoflix</t>
         </is>
@@ -3074,17 +2994,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
         <is>
           <t>Punkt.PRERADOVIC</t>
         </is>
@@ -3099,7 +3016,7 @@
           <t>157.000</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@punkt.preradovic3208</t>
         </is>
@@ -3124,17 +3041,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>Ignaz Bearth</t>
         </is>
@@ -3149,7 +3063,7 @@
           <t>157.000</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@IgnazBearthSchweiz</t>
         </is>
@@ -3174,17 +3088,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>Stein-Zeit (Archiv)</t>
         </is>
@@ -3199,7 +3110,7 @@
           <t>111.000</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@stein-zeit2355</t>
         </is>
@@ -3224,17 +3135,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>Eva Herman</t>
         </is>
@@ -3249,7 +3157,7 @@
           <t>80.100</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@EvaHermanOffiziell</t>
         </is>
@@ -3274,17 +3182,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>Samuel Eckert</t>
         </is>
@@ -3299,7 +3204,7 @@
           <t>74.400</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@SEyoutube</t>
         </is>
@@ -3324,17 +3229,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>Manova</t>
         </is>
@@ -3349,7 +3251,7 @@
           <t>68.000</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@Manova_Magazin</t>
         </is>
@@ -3374,17 +3276,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>Ulrike Guérot</t>
         </is>
@@ -3399,7 +3298,7 @@
           <t>64.400</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@UlrikeGuérot-Official</t>
         </is>
@@ -3424,17 +3323,14 @@
           <t>Alternative Medien &amp; Gesellschaft</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>Stefan Magnet</t>
         </is>
@@ -3449,7 +3345,7 @@
           <t>59.100</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@StefanMagnet</t>
         </is>
@@ -3488,7 +3384,7 @@
       <c r="L59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>BITTEL TV</t>
         </is>
@@ -3503,7 +3399,7 @@
           <t>49.500</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@bittel_tv</t>
         </is>
@@ -3543,6 +3439,126 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L60"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A54" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A55" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A56" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A57" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A58" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId118"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Kanalliste: Matthias Langwasser ergänzt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U8rX9WoPvch1isV4z66GEi
</commit_message>
<xml_diff>
--- a/recherche/youtube-kanaele-podcast-gaeste.xlsx
+++ b/recherche/youtube-kanaele-podcast-gaeste.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3436,6 +3436,56 @@
       </c>
       <c r="K60" s="2" t="inlineStr"/>
       <c r="L60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Matthias Langwasser</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Matthias Langwasser</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>147.000</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@MatthiasLangwasserKanal</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>aloha@matthias-langwasser.com</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>matthias-langwasser.de/kontakt</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Wöchentliche Interviews, Bewusstsein, Gesundheit, Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Bewusstsein &amp; Spiritualität</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L60"/>
@@ -3558,6 +3608,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId117"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A61" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId120"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>